<commit_message>
v0.9.65: convert \dontrun @examples to runnable/\donttest on community; add community 16th column JobSatisfaction (jdeclare_udm dirty-arrival demo); fix two jplot S3 message examples; generator JeffsStatTools->jstats
</commit_message>
<xml_diff>
--- a/inst/extdata/community_excel.xlsx
+++ b/inst/extdata/community_excel.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O101"/>
+  <dimension ref="A1:P101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -430,6 +430,11 @@
           <t>Environment5</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>JobSatisfaction</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -479,6 +484,9 @@
       <c r="O2">
         <v>4</v>
       </c>
+      <c r="P2">
+        <v>5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -528,6 +536,9 @@
       <c r="O3">
         <v>4</v>
       </c>
+      <c r="P3">
+        <v>-98</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -577,6 +588,9 @@
       <c r="O4">
         <v>4</v>
       </c>
+      <c r="P4">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -626,6 +640,9 @@
       <c r="O5">
         <v>1</v>
       </c>
+      <c r="P5">
+        <v>7</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -675,6 +692,9 @@
       <c r="O6">
         <v>4</v>
       </c>
+      <c r="P6">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -724,6 +744,9 @@
       <c r="O7">
         <v>5</v>
       </c>
+      <c r="P7">
+        <v>4</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -773,6 +796,9 @@
       <c r="O8">
         <v>1</v>
       </c>
+      <c r="P8">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -822,6 +848,9 @@
       <c r="O9">
         <v>5</v>
       </c>
+      <c r="P9">
+        <v>9</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -871,6 +900,9 @@
       <c r="O10">
         <v>5</v>
       </c>
+      <c r="P10">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -920,6 +952,9 @@
       <c r="O11">
         <v>1</v>
       </c>
+      <c r="P11">
+        <v>8</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -969,6 +1004,9 @@
       <c r="O12">
         <v>3</v>
       </c>
+      <c r="P12">
+        <v>6</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1018,6 +1056,9 @@
       <c r="O13">
         <v>5</v>
       </c>
+      <c r="P13">
+        <v>4</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1067,6 +1108,9 @@
       <c r="O14">
         <v>3</v>
       </c>
+      <c r="P14">
+        <v>6</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1116,6 +1160,9 @@
       <c r="O15">
         <v>3</v>
       </c>
+      <c r="P15">
+        <v>8</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1165,6 +1212,9 @@
       <c r="O16">
         <v>4</v>
       </c>
+      <c r="P16">
+        <v>7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1214,6 +1264,9 @@
       <c r="O17">
         <v>5</v>
       </c>
+      <c r="P17">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1263,6 +1316,9 @@
       <c r="O18">
         <v>5</v>
       </c>
+      <c r="P18">
+        <v>4</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1312,6 +1368,9 @@
       <c r="O19">
         <v>2</v>
       </c>
+      <c r="P19">
+        <v>8</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1361,6 +1420,9 @@
       <c r="O20">
         <v>3</v>
       </c>
+      <c r="P20">
+        <v>5</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1410,6 +1472,9 @@
       <c r="O21">
         <v>1</v>
       </c>
+      <c r="P21">
+        <v>4</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1459,6 +1524,9 @@
       <c r="O22">
         <v>1</v>
       </c>
+      <c r="P22">
+        <v>-98</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1508,6 +1576,9 @@
       <c r="O23">
         <v>1</v>
       </c>
+      <c r="P23">
+        <v>5</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1557,6 +1628,9 @@
       <c r="O24">
         <v>1</v>
       </c>
+      <c r="P24">
+        <v>-99</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1606,6 +1680,9 @@
       <c r="O25">
         <v>3</v>
       </c>
+      <c r="P25">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1655,6 +1732,9 @@
       <c r="O26">
         <v>1</v>
       </c>
+      <c r="P26">
+        <v>10</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1704,6 +1784,9 @@
       <c r="O27">
         <v>5</v>
       </c>
+      <c r="P27">
+        <v>6</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1753,6 +1836,9 @@
       <c r="O28">
         <v>3</v>
       </c>
+      <c r="P28">
+        <v>7</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1802,6 +1888,9 @@
       <c r="O29">
         <v>1</v>
       </c>
+      <c r="P29">
+        <v>9</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1851,6 +1940,9 @@
       <c r="O30">
         <v>1</v>
       </c>
+      <c r="P30">
+        <v>5</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1900,6 +1992,9 @@
       <c r="O31">
         <v>4</v>
       </c>
+      <c r="P31">
+        <v>5</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1949,6 +2044,9 @@
       <c r="O32">
         <v>2</v>
       </c>
+      <c r="P32">
+        <v>3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1998,6 +2096,9 @@
       <c r="O33">
         <v>5</v>
       </c>
+      <c r="P33">
+        <v>7</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2047,6 +2148,9 @@
       <c r="O34">
         <v>4</v>
       </c>
+      <c r="P34">
+        <v>6</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2096,6 +2200,9 @@
       <c r="O35">
         <v>3</v>
       </c>
+      <c r="P35">
+        <v>-99</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2145,6 +2252,9 @@
       <c r="O36">
         <v>3</v>
       </c>
+      <c r="P36">
+        <v>2</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2194,6 +2304,9 @@
       <c r="O37">
         <v>3</v>
       </c>
+      <c r="P37">
+        <v>5</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2243,6 +2356,9 @@
       <c r="O38">
         <v>5</v>
       </c>
+      <c r="P38">
+        <v>5</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2292,6 +2408,9 @@
       <c r="O39">
         <v>2</v>
       </c>
+      <c r="P39">
+        <v>4</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2341,6 +2460,9 @@
       <c r="O40">
         <v>1</v>
       </c>
+      <c r="P40">
+        <v>6</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2390,6 +2512,9 @@
       <c r="O41">
         <v>3</v>
       </c>
+      <c r="P41">
+        <v>-99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2439,6 +2564,9 @@
       <c r="O42">
         <v>1</v>
       </c>
+      <c r="P42">
+        <v>5</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2488,6 +2616,9 @@
       <c r="O43">
         <v>1</v>
       </c>
+      <c r="P43">
+        <v>6</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2537,6 +2668,9 @@
       <c r="O44">
         <v>1</v>
       </c>
+      <c r="P44">
+        <v>4</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2586,6 +2720,9 @@
       <c r="O45">
         <v>4</v>
       </c>
+      <c r="P45">
+        <v>3</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2635,6 +2772,9 @@
       <c r="O46">
         <v>2</v>
       </c>
+      <c r="P46">
+        <v>5</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2684,6 +2824,9 @@
       <c r="O47">
         <v>1</v>
       </c>
+      <c r="P47">
+        <v>-98</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2733,6 +2876,9 @@
       <c r="O48">
         <v>5</v>
       </c>
+      <c r="P48">
+        <v>5</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2782,6 +2928,9 @@
       <c r="O49">
         <v>5</v>
       </c>
+      <c r="P49">
+        <v>3</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2831,6 +2980,9 @@
       <c r="O50">
         <v>5</v>
       </c>
+      <c r="P50">
+        <v>7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2880,6 +3032,9 @@
       <c r="O51">
         <v>4</v>
       </c>
+      <c r="P51">
+        <v>7</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2929,6 +3084,9 @@
       <c r="O52">
         <v>2</v>
       </c>
+      <c r="P52">
+        <v>3</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2978,6 +3136,9 @@
       <c r="O53">
         <v>3</v>
       </c>
+      <c r="P53">
+        <v>6</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3027,6 +3188,9 @@
       <c r="O54">
         <v>5</v>
       </c>
+      <c r="P54">
+        <v>6</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3076,6 +3240,9 @@
       <c r="O55">
         <v>1</v>
       </c>
+      <c r="P55">
+        <v>8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3125,6 +3292,9 @@
       <c r="O56">
         <v>2</v>
       </c>
+      <c r="P56">
+        <v>7</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3174,6 +3344,9 @@
       <c r="O57">
         <v>1</v>
       </c>
+      <c r="P57">
+        <v>4</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3223,6 +3396,9 @@
       <c r="O58">
         <v>1</v>
       </c>
+      <c r="P58">
+        <v>7</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3272,6 +3448,9 @@
       <c r="O59">
         <v>4</v>
       </c>
+      <c r="P59">
+        <v>5</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3321,6 +3500,9 @@
       <c r="O60">
         <v>3</v>
       </c>
+      <c r="P60">
+        <v>6</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3370,6 +3552,9 @@
       <c r="O61">
         <v>2</v>
       </c>
+      <c r="P61">
+        <v>5</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3419,6 +3604,9 @@
       <c r="O62">
         <v>2</v>
       </c>
+      <c r="P62">
+        <v>4</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3468,6 +3656,9 @@
       <c r="O63">
         <v>3</v>
       </c>
+      <c r="P63">
+        <v>9</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3517,6 +3708,9 @@
       <c r="O64">
         <v>1</v>
       </c>
+      <c r="P64">
+        <v>8</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3566,6 +3760,9 @@
       <c r="O65">
         <v>4</v>
       </c>
+      <c r="P65">
+        <v>4</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3615,6 +3812,9 @@
       <c r="O66">
         <v>1</v>
       </c>
+      <c r="P66">
+        <v>4</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3664,6 +3864,9 @@
       <c r="O67">
         <v>2</v>
       </c>
+      <c r="P67">
+        <v>4</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3713,6 +3916,9 @@
       <c r="O68">
         <v>1</v>
       </c>
+      <c r="P68">
+        <v>8</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3762,6 +3968,9 @@
       <c r="O69">
         <v>3</v>
       </c>
+      <c r="P69">
+        <v>6</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3811,6 +4020,9 @@
       <c r="O70">
         <v>5</v>
       </c>
+      <c r="P70">
+        <v>5</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3860,6 +4072,9 @@
       <c r="O71">
         <v>3</v>
       </c>
+      <c r="P71">
+        <v>5</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3909,6 +4124,9 @@
       <c r="O72">
         <v>2</v>
       </c>
+      <c r="P72">
+        <v>8</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3958,6 +4176,9 @@
       <c r="O73">
         <v>1</v>
       </c>
+      <c r="P73">
+        <v>5</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4007,6 +4228,9 @@
       <c r="O74">
         <v>4</v>
       </c>
+      <c r="P74">
+        <v>3</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4056,6 +4280,9 @@
       <c r="O75">
         <v>3</v>
       </c>
+      <c r="P75">
+        <v>5</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4105,6 +4332,9 @@
       <c r="O76">
         <v>3</v>
       </c>
+      <c r="P76">
+        <v>9</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4154,6 +4384,9 @@
       <c r="O77">
         <v>1</v>
       </c>
+      <c r="P77">
+        <v>6</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4203,6 +4436,9 @@
       <c r="O78">
         <v>4</v>
       </c>
+      <c r="P78">
+        <v>8</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4252,6 +4488,9 @@
       <c r="O79">
         <v>2</v>
       </c>
+      <c r="P79">
+        <v>4</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4301,6 +4540,9 @@
       <c r="O80">
         <v>1</v>
       </c>
+      <c r="P80">
+        <v>2</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4350,6 +4592,9 @@
       <c r="O81">
         <v>1</v>
       </c>
+      <c r="P81">
+        <v>6</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4399,6 +4644,9 @@
       <c r="O82">
         <v>4</v>
       </c>
+      <c r="P82">
+        <v>8</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4448,6 +4696,9 @@
       <c r="O83">
         <v>5</v>
       </c>
+      <c r="P83">
+        <v>9</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4497,6 +4748,9 @@
       <c r="O84">
         <v>3</v>
       </c>
+      <c r="P84">
+        <v>8</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4546,6 +4800,9 @@
       <c r="O85">
         <v>4</v>
       </c>
+      <c r="P85">
+        <v>5</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4595,6 +4852,9 @@
       <c r="O86">
         <v>5</v>
       </c>
+      <c r="P86">
+        <v>-99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4644,6 +4904,9 @@
       <c r="O87">
         <v>1</v>
       </c>
+      <c r="P87">
+        <v>7</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4693,6 +4956,9 @@
       <c r="O88">
         <v>4</v>
       </c>
+      <c r="P88">
+        <v>6</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4742,6 +5008,9 @@
       <c r="O89">
         <v>3</v>
       </c>
+      <c r="P89">
+        <v>9</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4791,6 +5060,9 @@
       <c r="O90">
         <v>2</v>
       </c>
+      <c r="P90">
+        <v>7</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4840,6 +5112,9 @@
       <c r="O91">
         <v>3</v>
       </c>
+      <c r="P91">
+        <v>7</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4889,6 +5164,9 @@
       <c r="O92">
         <v>5</v>
       </c>
+      <c r="P92">
+        <v>3</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4938,6 +5216,9 @@
       <c r="O93">
         <v>4</v>
       </c>
+      <c r="P93">
+        <v>6</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4987,6 +5268,9 @@
       <c r="O94">
         <v>5</v>
       </c>
+      <c r="P94">
+        <v>7</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5036,6 +5320,9 @@
       <c r="O95">
         <v>4</v>
       </c>
+      <c r="P95">
+        <v>7</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5085,6 +5372,9 @@
       <c r="O96">
         <v>5</v>
       </c>
+      <c r="P96">
+        <v>7</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5134,6 +5424,9 @@
       <c r="O97">
         <v>2</v>
       </c>
+      <c r="P97">
+        <v>7</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5183,6 +5476,9 @@
       <c r="O98">
         <v>4</v>
       </c>
+      <c r="P98">
+        <v>5</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5232,6 +5528,9 @@
       <c r="O99">
         <v>4</v>
       </c>
+      <c r="P99">
+        <v>10</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5281,6 +5580,9 @@
       <c r="O100">
         <v>4</v>
       </c>
+      <c r="P100">
+        <v>7</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5329,6 +5631,9 @@
       </c>
       <c r="O101">
         <v>5</v>
+      </c>
+      <c r="P101">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v0.9.68: clinic second shipped dataset built (community trimmed to 15 cols); Rules K/L + mv fixes (M2 Option-B revert, jalpha Rule E, advisory blank line); javg/jsum headline mean + assign-reminder; Variable Labels = alignment
</commit_message>
<xml_diff>
--- a/inst/extdata/community_excel.xlsx
+++ b/inst/extdata/community_excel.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P101"/>
+  <dimension ref="A1:O101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -430,11 +430,6 @@
           <t>Environment5</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>JobSatisfaction</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -484,9 +479,6 @@
       <c r="O2">
         <v>4</v>
       </c>
-      <c r="P2">
-        <v>5</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -536,9 +528,6 @@
       <c r="O3">
         <v>4</v>
       </c>
-      <c r="P3">
-        <v>-98</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -588,9 +577,6 @@
       <c r="O4">
         <v>4</v>
       </c>
-      <c r="P4">
-        <v>5</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -640,9 +626,6 @@
       <c r="O5">
         <v>1</v>
       </c>
-      <c r="P5">
-        <v>7</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -692,9 +675,6 @@
       <c r="O6">
         <v>4</v>
       </c>
-      <c r="P6">
-        <v>4</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -744,9 +724,6 @@
       <c r="O7">
         <v>5</v>
       </c>
-      <c r="P7">
-        <v>4</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -796,9 +773,6 @@
       <c r="O8">
         <v>1</v>
       </c>
-      <c r="P8">
-        <v>5</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -848,9 +822,6 @@
       <c r="O9">
         <v>5</v>
       </c>
-      <c r="P9">
-        <v>9</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -900,9 +871,6 @@
       <c r="O10">
         <v>5</v>
       </c>
-      <c r="P10">
-        <v>6</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -952,9 +920,6 @@
       <c r="O11">
         <v>1</v>
       </c>
-      <c r="P11">
-        <v>8</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1004,9 +969,6 @@
       <c r="O12">
         <v>3</v>
       </c>
-      <c r="P12">
-        <v>6</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1056,9 +1018,6 @@
       <c r="O13">
         <v>5</v>
       </c>
-      <c r="P13">
-        <v>4</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1108,9 +1067,6 @@
       <c r="O14">
         <v>3</v>
       </c>
-      <c r="P14">
-        <v>6</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1160,9 +1116,6 @@
       <c r="O15">
         <v>3</v>
       </c>
-      <c r="P15">
-        <v>8</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1212,9 +1165,6 @@
       <c r="O16">
         <v>4</v>
       </c>
-      <c r="P16">
-        <v>7</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1264,9 +1214,6 @@
       <c r="O17">
         <v>5</v>
       </c>
-      <c r="P17">
-        <v>6</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1316,9 +1263,6 @@
       <c r="O18">
         <v>5</v>
       </c>
-      <c r="P18">
-        <v>4</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1368,9 +1312,6 @@
       <c r="O19">
         <v>2</v>
       </c>
-      <c r="P19">
-        <v>8</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1420,9 +1361,6 @@
       <c r="O20">
         <v>3</v>
       </c>
-      <c r="P20">
-        <v>5</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1472,9 +1410,6 @@
       <c r="O21">
         <v>1</v>
       </c>
-      <c r="P21">
-        <v>4</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1524,9 +1459,6 @@
       <c r="O22">
         <v>1</v>
       </c>
-      <c r="P22">
-        <v>-98</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1576,9 +1508,6 @@
       <c r="O23">
         <v>1</v>
       </c>
-      <c r="P23">
-        <v>5</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1628,9 +1557,6 @@
       <c r="O24">
         <v>1</v>
       </c>
-      <c r="P24">
-        <v>-99</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1680,9 +1606,6 @@
       <c r="O25">
         <v>3</v>
       </c>
-      <c r="P25">
-        <v>5</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1732,9 +1655,6 @@
       <c r="O26">
         <v>1</v>
       </c>
-      <c r="P26">
-        <v>10</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1784,9 +1704,6 @@
       <c r="O27">
         <v>5</v>
       </c>
-      <c r="P27">
-        <v>6</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1836,9 +1753,6 @@
       <c r="O28">
         <v>3</v>
       </c>
-      <c r="P28">
-        <v>7</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1888,9 +1802,6 @@
       <c r="O29">
         <v>1</v>
       </c>
-      <c r="P29">
-        <v>9</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1940,9 +1851,6 @@
       <c r="O30">
         <v>1</v>
       </c>
-      <c r="P30">
-        <v>5</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1992,9 +1900,6 @@
       <c r="O31">
         <v>4</v>
       </c>
-      <c r="P31">
-        <v>5</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2044,9 +1949,6 @@
       <c r="O32">
         <v>2</v>
       </c>
-      <c r="P32">
-        <v>3</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2096,9 +1998,6 @@
       <c r="O33">
         <v>5</v>
       </c>
-      <c r="P33">
-        <v>7</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2148,9 +2047,6 @@
       <c r="O34">
         <v>4</v>
       </c>
-      <c r="P34">
-        <v>6</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2200,9 +2096,6 @@
       <c r="O35">
         <v>3</v>
       </c>
-      <c r="P35">
-        <v>-99</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2252,9 +2145,6 @@
       <c r="O36">
         <v>3</v>
       </c>
-      <c r="P36">
-        <v>2</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2304,9 +2194,6 @@
       <c r="O37">
         <v>3</v>
       </c>
-      <c r="P37">
-        <v>5</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2356,9 +2243,6 @@
       <c r="O38">
         <v>5</v>
       </c>
-      <c r="P38">
-        <v>5</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2408,9 +2292,6 @@
       <c r="O39">
         <v>2</v>
       </c>
-      <c r="P39">
-        <v>4</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2460,9 +2341,6 @@
       <c r="O40">
         <v>1</v>
       </c>
-      <c r="P40">
-        <v>6</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2512,9 +2390,6 @@
       <c r="O41">
         <v>3</v>
       </c>
-      <c r="P41">
-        <v>-99</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2564,9 +2439,6 @@
       <c r="O42">
         <v>1</v>
       </c>
-      <c r="P42">
-        <v>5</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2616,9 +2488,6 @@
       <c r="O43">
         <v>1</v>
       </c>
-      <c r="P43">
-        <v>6</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2668,9 +2537,6 @@
       <c r="O44">
         <v>1</v>
       </c>
-      <c r="P44">
-        <v>4</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2720,9 +2586,6 @@
       <c r="O45">
         <v>4</v>
       </c>
-      <c r="P45">
-        <v>3</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2772,9 +2635,6 @@
       <c r="O46">
         <v>2</v>
       </c>
-      <c r="P46">
-        <v>5</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2824,9 +2684,6 @@
       <c r="O47">
         <v>1</v>
       </c>
-      <c r="P47">
-        <v>-98</v>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2876,9 +2733,6 @@
       <c r="O48">
         <v>5</v>
       </c>
-      <c r="P48">
-        <v>5</v>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2928,9 +2782,6 @@
       <c r="O49">
         <v>5</v>
       </c>
-      <c r="P49">
-        <v>3</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2980,9 +2831,6 @@
       <c r="O50">
         <v>5</v>
       </c>
-      <c r="P50">
-        <v>7</v>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3032,9 +2880,6 @@
       <c r="O51">
         <v>4</v>
       </c>
-      <c r="P51">
-        <v>7</v>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3084,9 +2929,6 @@
       <c r="O52">
         <v>2</v>
       </c>
-      <c r="P52">
-        <v>3</v>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3136,9 +2978,6 @@
       <c r="O53">
         <v>3</v>
       </c>
-      <c r="P53">
-        <v>6</v>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3188,9 +3027,6 @@
       <c r="O54">
         <v>5</v>
       </c>
-      <c r="P54">
-        <v>6</v>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3240,9 +3076,6 @@
       <c r="O55">
         <v>1</v>
       </c>
-      <c r="P55">
-        <v>8</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3292,9 +3125,6 @@
       <c r="O56">
         <v>2</v>
       </c>
-      <c r="P56">
-        <v>7</v>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3344,9 +3174,6 @@
       <c r="O57">
         <v>1</v>
       </c>
-      <c r="P57">
-        <v>4</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3396,9 +3223,6 @@
       <c r="O58">
         <v>1</v>
       </c>
-      <c r="P58">
-        <v>7</v>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3448,9 +3272,6 @@
       <c r="O59">
         <v>4</v>
       </c>
-      <c r="P59">
-        <v>5</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3500,9 +3321,6 @@
       <c r="O60">
         <v>3</v>
       </c>
-      <c r="P60">
-        <v>6</v>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3552,9 +3370,6 @@
       <c r="O61">
         <v>2</v>
       </c>
-      <c r="P61">
-        <v>5</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3604,9 +3419,6 @@
       <c r="O62">
         <v>2</v>
       </c>
-      <c r="P62">
-        <v>4</v>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3656,9 +3468,6 @@
       <c r="O63">
         <v>3</v>
       </c>
-      <c r="P63">
-        <v>9</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3708,9 +3517,6 @@
       <c r="O64">
         <v>1</v>
       </c>
-      <c r="P64">
-        <v>8</v>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3760,9 +3566,6 @@
       <c r="O65">
         <v>4</v>
       </c>
-      <c r="P65">
-        <v>4</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3812,9 +3615,6 @@
       <c r="O66">
         <v>1</v>
       </c>
-      <c r="P66">
-        <v>4</v>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3864,9 +3664,6 @@
       <c r="O67">
         <v>2</v>
       </c>
-      <c r="P67">
-        <v>4</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3916,9 +3713,6 @@
       <c r="O68">
         <v>1</v>
       </c>
-      <c r="P68">
-        <v>8</v>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3968,9 +3762,6 @@
       <c r="O69">
         <v>3</v>
       </c>
-      <c r="P69">
-        <v>6</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4020,9 +3811,6 @@
       <c r="O70">
         <v>5</v>
       </c>
-      <c r="P70">
-        <v>5</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4072,9 +3860,6 @@
       <c r="O71">
         <v>3</v>
       </c>
-      <c r="P71">
-        <v>5</v>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4124,9 +3909,6 @@
       <c r="O72">
         <v>2</v>
       </c>
-      <c r="P72">
-        <v>8</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4176,9 +3958,6 @@
       <c r="O73">
         <v>1</v>
       </c>
-      <c r="P73">
-        <v>5</v>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4228,9 +4007,6 @@
       <c r="O74">
         <v>4</v>
       </c>
-      <c r="P74">
-        <v>3</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4280,9 +4056,6 @@
       <c r="O75">
         <v>3</v>
       </c>
-      <c r="P75">
-        <v>5</v>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4332,9 +4105,6 @@
       <c r="O76">
         <v>3</v>
       </c>
-      <c r="P76">
-        <v>9</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4384,9 +4154,6 @@
       <c r="O77">
         <v>1</v>
       </c>
-      <c r="P77">
-        <v>6</v>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4436,9 +4203,6 @@
       <c r="O78">
         <v>4</v>
       </c>
-      <c r="P78">
-        <v>8</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4488,9 +4252,6 @@
       <c r="O79">
         <v>2</v>
       </c>
-      <c r="P79">
-        <v>4</v>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4540,9 +4301,6 @@
       <c r="O80">
         <v>1</v>
       </c>
-      <c r="P80">
-        <v>2</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4592,9 +4350,6 @@
       <c r="O81">
         <v>1</v>
       </c>
-      <c r="P81">
-        <v>6</v>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4644,9 +4399,6 @@
       <c r="O82">
         <v>4</v>
       </c>
-      <c r="P82">
-        <v>8</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4696,9 +4448,6 @@
       <c r="O83">
         <v>5</v>
       </c>
-      <c r="P83">
-        <v>9</v>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4748,9 +4497,6 @@
       <c r="O84">
         <v>3</v>
       </c>
-      <c r="P84">
-        <v>8</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4800,9 +4546,6 @@
       <c r="O85">
         <v>4</v>
       </c>
-      <c r="P85">
-        <v>5</v>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4852,9 +4595,6 @@
       <c r="O86">
         <v>5</v>
       </c>
-      <c r="P86">
-        <v>-99</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4904,9 +4644,6 @@
       <c r="O87">
         <v>1</v>
       </c>
-      <c r="P87">
-        <v>7</v>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4956,9 +4693,6 @@
       <c r="O88">
         <v>4</v>
       </c>
-      <c r="P88">
-        <v>6</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5008,9 +4742,6 @@
       <c r="O89">
         <v>3</v>
       </c>
-      <c r="P89">
-        <v>9</v>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5060,9 +4791,6 @@
       <c r="O90">
         <v>2</v>
       </c>
-      <c r="P90">
-        <v>7</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5112,9 +4840,6 @@
       <c r="O91">
         <v>3</v>
       </c>
-      <c r="P91">
-        <v>7</v>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5164,9 +4889,6 @@
       <c r="O92">
         <v>5</v>
       </c>
-      <c r="P92">
-        <v>3</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5216,9 +4938,6 @@
       <c r="O93">
         <v>4</v>
       </c>
-      <c r="P93">
-        <v>6</v>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5268,9 +4987,6 @@
       <c r="O94">
         <v>5</v>
       </c>
-      <c r="P94">
-        <v>7</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5320,9 +5036,6 @@
       <c r="O95">
         <v>4</v>
       </c>
-      <c r="P95">
-        <v>7</v>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5372,9 +5085,6 @@
       <c r="O96">
         <v>5</v>
       </c>
-      <c r="P96">
-        <v>7</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5424,9 +5134,6 @@
       <c r="O97">
         <v>2</v>
       </c>
-      <c r="P97">
-        <v>7</v>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5476,9 +5183,6 @@
       <c r="O98">
         <v>4</v>
       </c>
-      <c r="P98">
-        <v>5</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5528,9 +5232,6 @@
       <c r="O99">
         <v>4</v>
       </c>
-      <c r="P99">
-        <v>10</v>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5580,9 +5281,6 @@
       <c r="O100">
         <v>4</v>
       </c>
-      <c r="P100">
-        <v>7</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5631,9 +5329,6 @@
       </c>
       <c r="O101">
         <v>5</v>
-      </c>
-      <c r="P101">
-        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>